<commit_message>
add mcf temperature zone lookup to common input functions
</commit_message>
<xml_diff>
--- a/Excel/Common_v02.xlsx
+++ b/Excel/Common_v02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E6FEFB5-2EBA-45CB-AFD0-37A0943ACDC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF39F33-F015-47E3-B46D-EB4BA39A554C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30" yWindow="105" windowWidth="28875" windowHeight="16890" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="0" yWindow="390" windowWidth="28800" windowHeight="16890" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="3" r:id="rId1"/>
@@ -37,6 +37,8 @@
     <definedName name="Common_InputFunctions.getOverlappingReportingCycles">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingCycleStart, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, MONTH(_xlpm.ReportingCycleStart), _xlpm.d, DAY(_xlpm.ReportingCycleStart), _xlpm.PeriodEnd, _xlfn.LAMBDA(_xlpm.st, EDATE(_xlpm.st, 12) - 1), _xlpm.A, _xlpm.S - 365, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (_xlpm.PeriodEnd(DATE(_xlpm.ya, _xlpm.m, _xlpm.d)) &lt; _xlpm.S), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1)))</definedName>
     <definedName name="Common_InputFunctions.getOverlappingReportingPeriods">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingCycleStart, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, MONTH(_xlpm.ReportingCycleStart), _xlpm.d, DAY(_xlpm.ReportingCycleStart), _xlpm.PeriodEnd, _xlfn.LAMBDA(_xlpm.st, EDATE(_xlpm.st, 12) - 1), _xlpm.A, _xlpm.S - 365, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (_xlpm.PeriodEnd(DATE(_xlpm.ya, _xlpm.m, _xlpm.d)) &lt; _xlpm.S), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), _xlpm.n, MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1), _xlpm.yrs, _xlfn.SEQUENCE(_xlpm.n, 1, _xlpm.firstYear, 1), _xlpm.starts, DATE(_xlpm.yrs, _xlpm.m, _xlpm.d), _xlpm.ends, _xlfn.MAP(_xlpm.starts, _xlpm.PeriodEnd), _xlpm.tag, IF(_xlpm.starts = _xlpm.ReportingCycleStart, " (This reporting cycle)", ""), _xlpm.startsText, TEXT(_xlpm.starts, "dd mmm yyyy"), _xlpm.endsText, TEXT(_xlpm.ends, "dd mmm yyyy"), IF(_xlpm.n = 0, "", _xlfn.HSTACK(_xlpm.startsText &amp; " to " &amp; _xlpm.endsText &amp; _xlpm.tag))))</definedName>
     <definedName name="Common_InputFunctions.Utility_ConvertStateCommonNameToAbbreviation">_xlfn.LAMBDA(_xlpm.StateCommonName,_xlpm.StateCommonNameArray,_xlpm.StateAbbreviationArray, _xlfn.XLOOKUP(_xlpm.StateCommonName, _xlpm.StateCommonNameArray, _xlpm.StateAbbreviationArray, ""))</definedName>
+    <definedName name="Common_InputFunctions.Utility_DisplayArguments_1_2">_xlfn.LAMBDA(_xlpm.ArgumentsArray, _xlfn.CHOOSECOLS(_xlpm.ArgumentsArray, 1, 2))</definedName>
+    <definedName name="Common_InputFunctions.Utility_DisplayArguments_3_4">_xlfn.LAMBDA(_xlpm.ArgumentsArray, _xlfn.CHOOSECOLS(_xlpm.ArgumentsArray, 3, 4))</definedName>
     <definedName name="Common_InputFunctions.Utility_DisplayArrayInTable">_xlfn.LAMBDA(_xlpm.ArrayData,_xlpm.TableheaderCell,_xlpm.RowsBetweenHeaderandArray,_xlop.ColumnsBetweenHeaderAndArray, IFERROR(INDEX(_xlfn.UNIQUE(_xlpm.ArrayData), ROW() - Common_InputFunctions.Utility_GetArrayTableRowStartNumber(_xlpm.TableheaderCell, _xlpm.RowsBetweenHeaderandArray), COLUMN() - Common_InputFunctions.Utility_GetArrayTableColumnStartNumber(_xlpm.TableheaderCell) + IF(_xlfn.ISOMITTED(_xlpm.ColumnsBetweenHeaderAndArray), 1, _xlpm.ColumnsBetweenHeaderAndArray)), ""))</definedName>
     <definedName name="Common_InputFunctions.Utility_DisplayFunctionName">_xlfn.LAMBDA(_xlpm.Function, _xlfn.TEXTBEFORE(_xlfn.FORMULATEXT(_xlpm.Function), "("))</definedName>
     <definedName name="Common_InputFunctions.Utility_GetArrayTableColumnStartNumber">_xlfn.LAMBDA(_xlpm.TableHeaderCell, COLUMN(_xlpm.TableHeaderCell))</definedName>
@@ -48,6 +50,7 @@
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableNumber">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.LookupArray,_xlpm.ReturnArray, IF(ISNUMBER(_xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, "")), _xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, ""), 0))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableOneColumnAndHeader">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray, _xlfn.XLOOKUP(_xlpm.LookupValue1, _xlpm.LookupArray1, _xlfn.XLOOKUP(_xlpm.LookupValue2, _xlpm.LookupArray2, _xlpm.ReturnArray)))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableTwoColumns">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray, _xlfn.XLOOKUP(1, (_xlpm.LookupArray1 = _xlpm.LookupValue1) * (_xlpm.LookupArray2 = _xlpm.LookupValue2), _xlpm.ReturnArray, ""))</definedName>
+    <definedName name="Common_InputFunctions.Utility_SourceHyperlink">_xlfn.LAMBDA(_xlpm.TargetCell, _xlfn.LET(_xlpm.sh, _xlfn.TEXTAFTER(CELL("filename", _xlpm.TargetCell), "]"), _xlpm.addr, CELL("address", _xlpm.TargetCell), "#'" &amp; _xlpm.sh &amp; "'!" &amp; _xlpm.addr))</definedName>
     <definedName name="Common_InputFunctions.Utility_SplitStringIntoArray">_xlfn.LAMBDA(_xlpm.Cell,_xlpm.Delimiter,_xlop.CharacterToRemove1,_xlop.CharacterToRemove2, _xlfn.FILTERXML("&lt;t&gt;&lt;s&gt;" &amp; SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlpm.Cell, _xlpm.CharacterToRemove1, ""), _xlpm.CharacterToRemove2, ""), _xlpm.Delimiter, "&lt;/s&gt;&lt;s&gt;") &amp; "&lt;/s&gt;&lt;/t&gt;", "//s"))</definedName>
     <definedName name="Common_InputFunctions.Utility_SumQuantityFromCriteria">_xlfn.LAMBDA(_xlpm.Criteria1,_xlpm.Criteria1TypeArray,_xlpm.Quantity,_xlop.Multiplier,_xlop.Criteria2,_xlop.Criteria2Array, _xlfn.LET(_xlpm.multiplier, IF(_xlfn.ISOMITTED(_xlpm.Multiplier), 1, _xlpm.Multiplier), _xlpm.quantity, _xlpm.Quantity * _xlpm.multiplier, _xlpm.criteria1, --(_xlpm.Criteria1TypeArray = _xlpm.Criteria1), _xlpm.criteria2, IF(_xlfn.ISOMITTED(_xlpm.Criteria2), 1, --(_xlpm.Criteria2Array = _xlpm.Criteria2)), SUMPRODUCT(_xlpm.criteria1 * _xlpm.criteria2 * _xlpm.quantity)))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(9, 3, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State/Territory","Common Name","Abbreviation";"New South Wales","New South Wales","NSW";"Australian Capital Territory","ACT","ACT";"Victoria","Victoria","VIC";"Queensland","Queensland","QLD";"South Australia","South Australia","SA";"Western Australia","Western Australia","WA";"Tasmania","Tasmania","TAS";"Northern Territory","Northern Territory","NT"}, _xlpm.r, _xlpm.c))))</definedName>
@@ -984,7 +987,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="26" fillId="4" borderId="0" xfId="8">
       <alignment horizontal="left" vertical="center"/>
@@ -1021,10 +1024,7 @@
     <xf numFmtId="0" fontId="27" fillId="4" borderId="0" xfId="54">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2901,7 +2901,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="825" row="4">
+  <wetp:taskpane dockstate="right" visibility="0" width="849" row="4">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -5558,117 +5558,117 @@
       </c>
     </row>
     <row r="231" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D231" s="14" t="s">
+      <c r="D231" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="E231" s="14" t="s">
+      <c r="E231" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="F231" s="15" t="s">
+      <c r="F231" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="G231" s="14" t="s">
+      <c r="G231" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="H231" s="14" t="s">
+      <c r="H231" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="I231" s="14" t="s">
+      <c r="I231" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="J231" s="14" t="s">
+      <c r="J231" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="K231" s="14" t="s">
+      <c r="K231" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="L231" s="14" t="s">
+      <c r="L231" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="M231" s="14" t="s">
+      <c r="M231" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="N231" s="14" t="s">
+      <c r="N231" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="O231" s="14" t="s">
+      <c r="O231" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="P231" s="14" t="s">
+      <c r="P231" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="Q231" s="14" t="s">
+      <c r="Q231" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="R231" s="14" t="s">
+      <c r="R231" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="S231" s="14" t="s">
+      <c r="S231" s="11" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="232" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D232" s="14" t="str" cm="1">
+      <c r="D232" s="11" t="str" cm="1">
         <f t="array" ref="D232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Cool</v>
       </c>
-      <c r="E232" s="14" t="str" cm="1">
+      <c r="E232" s="11" t="str" cm="1">
         <f t="array" ref="E232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>≤10</v>
       </c>
-      <c r="F232" s="14" cm="1">
+      <c r="F232" s="11" cm="1">
         <f t="array" ref="F232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>0.66</v>
       </c>
-      <c r="G232" s="14" cm="1">
+      <c r="G232" s="11" cm="1">
         <f t="array" ref="G232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>0.1</v>
       </c>
-      <c r="H232" s="14" cm="1">
+      <c r="H232" s="11" cm="1">
         <f t="array" ref="H232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>0.1</v>
       </c>
-      <c r="I232" s="14" cm="1">
+      <c r="I232" s="11" cm="1">
         <f t="array" ref="I232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>1E-3</v>
       </c>
-      <c r="J232" s="14" cm="1">
+      <c r="J232" s="11" cm="1">
         <f t="array" ref="J232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="K232" s="14" cm="1">
+      <c r="K232" s="11" cm="1">
         <f t="array" ref="K232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>0.02</v>
       </c>
-      <c r="L232" s="14" cm="1">
+      <c r="L232" s="11" cm="1">
         <f t="array" ref="L232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>0.03</v>
       </c>
-      <c r="M232" s="14" cm="1">
+      <c r="M232" s="11" cm="1">
         <f t="array" ref="M232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>0.04</v>
       </c>
-      <c r="N232" s="14" cm="1">
+      <c r="N232" s="11" cm="1">
         <f t="array" ref="N232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="O232" s="14" cm="1">
+      <c r="O232" s="11" cm="1">
         <f t="array" ref="O232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="P232" s="14" cm="1">
+      <c r="P232" s="11" cm="1">
         <f t="array" ref="P232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>0</v>
       </c>
-      <c r="Q232" s="14" cm="1">
+      <c r="Q232" s="11" cm="1">
         <f t="array" ref="Q232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>0</v>
       </c>
-      <c r="R232" s="14" cm="1">
+      <c r="R232" s="11" cm="1">
         <f t="array" ref="R232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S232" s="14" cm="1">
+      <c r="S232" s="11" cm="1">
         <f t="array" ref="S232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>10</v>
       </c>
@@ -5734,7 +5734,7 @@
         <f t="array" ref="R233">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S233" s="14" cm="1">
+      <c r="S233" s="11" cm="1">
         <f t="array" ref="S233">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>11</v>
       </c>
@@ -5800,7 +5800,7 @@
         <f t="array" ref="R234">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S234" s="14" cm="1">
+      <c r="S234" s="11" cm="1">
         <f t="array" ref="S234">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>12</v>
       </c>
@@ -5866,7 +5866,7 @@
         <f t="array" ref="R235">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S235" s="14" cm="1">
+      <c r="S235" s="11" cm="1">
         <f t="array" ref="S235">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>13</v>
       </c>
@@ -5932,7 +5932,7 @@
         <f t="array" ref="R236">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S236" s="14" cm="1">
+      <c r="S236" s="11" cm="1">
         <f t="array" ref="S236">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>14</v>
       </c>
@@ -5998,7 +5998,7 @@
         <f t="array" ref="R237">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S237" s="14" cm="1">
+      <c r="S237" s="11" cm="1">
         <f t="array" ref="S237">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>15</v>
       </c>
@@ -6064,7 +6064,7 @@
         <f t="array" ref="R238">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S238" s="14" cm="1">
+      <c r="S238" s="11" cm="1">
         <f t="array" ref="S238">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>16</v>
       </c>
@@ -6130,7 +6130,7 @@
         <f t="array" ref="R239">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S239" s="14" cm="1">
+      <c r="S239" s="11" cm="1">
         <f t="array" ref="S239">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>17</v>
       </c>
@@ -6196,7 +6196,7 @@
         <f t="array" ref="R240">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S240" s="14" cm="1">
+      <c r="S240" s="11" cm="1">
         <f t="array" ref="S240">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>18</v>
       </c>
@@ -6262,7 +6262,7 @@
         <f t="array" ref="R241">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S241" s="14" cm="1">
+      <c r="S241" s="11" cm="1">
         <f t="array" ref="S241">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>19</v>
       </c>
@@ -6328,7 +6328,7 @@
         <f t="array" ref="R242">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S242" s="14" cm="1">
+      <c r="S242" s="11" cm="1">
         <f t="array" ref="S242">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>20</v>
       </c>
@@ -6394,7 +6394,7 @@
         <f t="array" ref="R243">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S243" s="14" cm="1">
+      <c r="S243" s="11" cm="1">
         <f t="array" ref="S243">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>21</v>
       </c>
@@ -6460,7 +6460,7 @@
         <f t="array" ref="R244">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S244" s="14" cm="1">
+      <c r="S244" s="11" cm="1">
         <f t="array" ref="S244">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>22</v>
       </c>
@@ -6526,7 +6526,7 @@
         <f t="array" ref="R245">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S245" s="14" cm="1">
+      <c r="S245" s="11" cm="1">
         <f t="array" ref="S245">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>23</v>
       </c>
@@ -6592,7 +6592,7 @@
         <f t="array" ref="R246">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S246" s="14" cm="1">
+      <c r="S246" s="11" cm="1">
         <f t="array" ref="S246">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>24</v>
       </c>
@@ -6658,7 +6658,7 @@
         <f t="array" ref="R247">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S247" s="14" cm="1">
+      <c r="S247" s="11" cm="1">
         <f t="array" ref="S247">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>25</v>
       </c>
@@ -6724,7 +6724,7 @@
         <f t="array" ref="R248">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S248" s="14" cm="1">
+      <c r="S248" s="11" cm="1">
         <f t="array" ref="S248">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>26</v>
       </c>
@@ -6790,7 +6790,7 @@
         <f t="array" ref="R249">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S249" s="14" cm="1">
+      <c r="S249" s="11" cm="1">
         <f t="array" ref="S249">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>27</v>
       </c>
@@ -6856,7 +6856,7 @@
         <f t="array" ref="R250">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="S250" s="14" cm="1">
+      <c r="S250" s="11" cm="1">
         <f t="array" ref="S250">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>28</v>
       </c>
@@ -6901,14 +6901,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7107,25 +7105,24 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAPAB0AD4APABzAD4AXAAiACAAJgBcAG4AIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFMAVQBCAFMAVABJAFQAVQBUAEUAKABDAGUAbABsACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEALABcACIAXAAiACkALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABEAGUAbABpAG0AaQB0AGUAcgAsAFwAIgA8AC8AcwA+ADwAcwA+AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAXAAiADwALwBzAD4APAAvAHQAPgBcACIALABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAvAC8AcwBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAGEAdgBnAFQAZQBtAHAALABhAHYAZwBSAGEAaQBuACwAZgByAG8AcwB0AEQAYQB5AHMALABlAGwAZQB2ACwAbQBhAHAAXwBwAGUAdAAsAFwAbgAgACAAIAAgAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACwAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkALABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUABFAFQAQQByAHIAYQB5ACwAbQBhAHgAUABFAFQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAD4APQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApADwAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAD4APQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApADwAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQA+AD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQA8AD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAD4APQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAPAA9AG0AYQBwAF8AcABlAHQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABQAEUAVABBAHIAcgBhAHkAKQA+AD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAPAA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAD4APQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABJAHQAZQBtAEEAcgByAGEAeQAsACAAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAQwByAGkAdABlAHIAaQBhADEALAAgAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5ACwAIABRAHUAYQBuAHQAaQB0AHkALAAgAFsATQB1AGwAdABpAHAAbABpAGUAcgBdACwAIABbAEMAcgBpAHQAZQByAGkAYQAyAF0ALABbAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQBdACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgATQB1AGwAdABpAHAAbABpAGUAcgApACwAMQAsAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsAFwAbgAgACAAIAAgAHEAdQBhAG4AdABpAHQAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACoATQB1AGwAdABpAHAAbABpAGUAcgAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMQApACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADIALABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAcgBpAHQAZQByAGkAYQAyACkALAAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADIAKQApACwAXABuACAAIAAgACAAUwBVAE0AUABSAE8ARABVAEMAVAAoAGMAcgBpAHQAZQByAGkAYQAxACoAYwByAGkAdABlAHIAaQBhADIAKgBxAHUAYQBuAHQAaQB0AHkAKQBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApADwAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AJwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAG4AZQB4AHQAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPABTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAD4ARQApACwAXABuACAAIAAgACAAIAAgACAAIABuACwATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAcgBzACwAUwBFAFEAVQBFAE4AQwBFACgAbgAsADEALABmAGkAcgBzAHQAWQBlAGEAcgAsADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMALABEAEEAVABFACgAeQByAHMALABtACwAZAApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzACwATQBBAFAAKABzAHQAYQByAHQAcwAsAFAAZQByAGkAbwBkAEUAbgBkACkALABcAG4AIAAgACAAIAAgACAAIAAgAHQAYQBnACwASQBGACgAcwB0AGEAcgB0AHMAPQBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXAAiACAAKABUAGgAaQBzACAAcgBlAHAAbwByAHQAaQBuAGcAIABjAHkAYwBsAGUAKQBcACIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzAFQAZQB4AHQALABUAEUAWABUACgAcwB0AGEAcgB0AHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzAFQAZQB4AHQALABUAEUAWABUACgAZQBuAGQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgACYAIABcACIAIAB0AG8AIABcACIAIAAmACAAZQBuAGQAcwBUAGUAeAB0ACAAJgAgAHQAYQBnACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQBcAG4APQBMAEEATQBCAEQAQQAoAEYAdQBuAGMAdABpAG8AbgAsACAAVABFAFgAVABCAEUARgBPAFIARQAoAEYATwBSAE0AVQBMAEEAVABFAFgAVAAoAEYAdQBuAGMAdABpAG8AbgApACwAIABcACIAKABcACIAKQApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5ACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkALABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAA9AFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACAAPQAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5AD0AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkAPQBJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkAPQBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAD4AMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAATQBNAFMALAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFwAbgAgACAAIAAgACAAIAAgACAATQBFAEQASQBBAE4AKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAPAB0AD4APABzAD4AXAAiACAAJgBcAG4AIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFMAVQBCAFMAVABJAFQAVQBUAEUAKABDAGUAbABsACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEALABcACIAXAAiACkALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABEAGUAbABpAG0AaQB0AGUAcgAsAFwAIgA8AC8AcwA+ADwAcwA+AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAXAAiADwALwBzAD4APAAvAHQAPgBcACIALABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAvAC8AcwBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAGEAdgBnAFQAZQBtAHAALABhAHYAZwBSAGEAaQBuACwAZgByAG8AcwB0AEQAYQB5AHMALABlAGwAZQB2ACwAbQBhAHAAXwBwAGUAdAAsAFwAbgAgACAAIAAgAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACwAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkALABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUABFAFQAQQByAHIAYQB5ACwAbQBhAHgAUABFAFQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAD4APQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApADwAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAD4APQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApADwAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQA+AD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQA8AD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAD4APQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAPAA9AG0AYQBwAF8AcABlAHQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABQAEUAVABBAHIAcgBhAHkAKQA+AD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAPAA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAD4APQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABJAHQAZQBtAEEAcgByAGEAeQAsACAAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAQwByAGkAdABlAHIAaQBhADEALAAgAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5ACwAIABRAHUAYQBuAHQAaQB0AHkALAAgAFsATQB1AGwAdABpAHAAbABpAGUAcgBdACwAIABbAEMAcgBpAHQAZQByAGkAYQAyAF0ALABbAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQBdACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgATQB1AGwAdABpAHAAbABpAGUAcgApACwAMQAsAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsAFwAbgAgACAAIAAgAHEAdQBhAG4AdABpAHQAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACoATQB1AGwAdABpAHAAbABpAGUAcgAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMQApACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADIALABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAcgBpAHQAZQByAGkAYQAyACkALAAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADIAKQApACwAXABuACAAIAAgACAAUwBVAE0AUABSAE8ARABVAEMAVAAoAGMAcgBpAHQAZQByAGkAYQAxACoAYwByAGkAdABlAHIAaQBhADIAKgBxAHUAYQBuAHQAaQB0AHkAKQBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApADwAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AJwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAG4AZQB4AHQAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPABTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAD4ARQApACwAXABuACAAIAAgACAAIAAgACAAIABuACwATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAcgBzACwAUwBFAFEAVQBFAE4AQwBFACgAbgAsADEALABmAGkAcgBzAHQAWQBlAGEAcgAsADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMALABEAEEAVABFACgAeQByAHMALABtACwAZAApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzACwATQBBAFAAKABzAHQAYQByAHQAcwAsAFAAZQByAGkAbwBkAEUAbgBkACkALABcAG4AIAAgACAAIAAgACAAIAAgAHQAYQBnACwASQBGACgAcwB0AGEAcgB0AHMAPQBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXAAiACAAKABUAGgAaQBzACAAcgBlAHAAbwByAHQAaQBuAGcAIABjAHkAYwBsAGUAKQBcACIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzAFQAZQB4AHQALABUAEUAWABUACgAcwB0AGEAcgB0AHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzAFQAZQB4AHQALABUAEUAWABUACgAZQBuAGQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgACYAIABcACIAIAB0AG8AIABcACIAIAAmACAAZQBuAGQAcwBUAGUAeAB0ACAAJgAgAHQAYQBnACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQBcAG4APQBMAEEATQBCAEQAQQAoAEYAdQBuAGMAdABpAG8AbgAsACAAVABFAFgAVABCAEUARgBPAFIARQAoAEYATwBSAE0AVQBMAEEAVABFAFgAVAAoAEYAdQBuAGMAdABpAG8AbgApACwAIABcACIAKABcACIAKQApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5ACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkALABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAA9AFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACAAPQAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5AD0AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkAPQBJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkAPQBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAD4AMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAJwBcACIAIAAmACAAcwBoACAAJgAgAFwAIgAnACEAXAAiACAAJgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEkATgAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBYACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAE0ATQBTACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7150,9 +7147,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
move notes away from climate zone lookup table
</commit_message>
<xml_diff>
--- a/Excel/Common_v02.xlsx
+++ b/Excel/Common_v02.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{480B05D6-AEA0-4B4C-B1A3-2ADE4CBF62B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CD6DD20-F011-445D-B09A-D8B6120FF91E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2970" yWindow="1590" windowWidth="28800" windowHeight="16890" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="1260" yWindow="1125" windowWidth="37140" windowHeight="20475" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="3" r:id="rId1"/>
@@ -213,7 +213,6 @@
     <definedName name="Step3">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1001,7 +1000,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="26" fillId="4" borderId="0" xfId="8">
       <alignment horizontal="left" vertical="center"/>
@@ -1039,9 +1038,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4410,31 +4406,31 @@
       </c>
       <c r="T97" s="11"/>
     </row>
-    <row r="98" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D98" s="12" t="str" cm="1">
-        <f t="array" ref="D98:D101">Common_SourceData.Common_SourceData_ClimateZones_Appendices()</f>
+    <row r="98" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D99" s="12" t="str" cm="1">
+        <f t="array" ref="D99:D102">Common_SourceData.Common_SourceData_ClimateZones_Appendices()</f>
         <v>Note:</v>
-      </c>
-    </row>
-    <row r="99" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D99" s="12" t="str">
-        <v>MAT = mean annual temperature</v>
       </c>
     </row>
     <row r="100" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D100" s="12" t="str">
-        <v>MAP = mean annual precipitation</v>
+        <v>MAT = mean annual temperature</v>
       </c>
     </row>
     <row r="101" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D101" s="12" t="str">
+        <v>MAP = mean annual precipitation</v>
+      </c>
+    </row>
+    <row r="102" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D102" s="12" t="str">
         <v>PET = potential evapotranspiration</v>
       </c>
     </row>
-    <row r="102" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D102" s="12"/>
-    </row>
-    <row r="103" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D103" s="12"/>
+    </row>
     <row r="104" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="105" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D105" s="5" t="str" cm="1">
@@ -6945,19 +6941,19 @@
       </c>
     </row>
     <row r="257" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D257" s="15" t="s">
+      <c r="D257" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="E257" s="15" t="s">
+      <c r="E257" s="11" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="258" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D258" s="15" t="str" cm="1">
+      <c r="D258" s="11" t="str" cm="1">
         <f t="array" ref="D258">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</f>
         <v>Wet climate zone</v>
       </c>
-      <c r="E258" s="15" cm="1">
+      <c r="E258" s="11" cm="1">
         <f t="array" ref="E258">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</f>
         <v>6.0000000000000001E-3</v>
       </c>
@@ -7013,17 +7009,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -7218,7 +7203,22 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAG4AZAAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIAByAGUAdAB1AHIAbgBlAGQAIAB0AG8AIAB0AGgAZQAgAHMAbwBpAGwAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUARgBOAGkAIAAmACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAJgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAPAB0AD4APABzAD4AXAAiACAAJgBcAG4AIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFMAVQBCAFMAVABJAFQAVQBUAEUAKABDAGUAbABsACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEALABcACIAXAAiACkALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABEAGUAbABpAG0AaQB0AGUAcgAsAFwAIgA8AC8AcwA+ADwAcwA+AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAXAAiADwALwBzAD4APAAvAHQAPgBcACIALABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAvAC8AcwBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAGEAdgBnAFQAZQBtAHAALABhAHYAZwBSAGEAaQBuACwAZgByAG8AcwB0AEQAYQB5AHMALABlAGwAZQB2ACwAbQBhAHAAXwBwAGUAdAAsAFwAbgAgACAAIAAgAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACwAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkALABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUABFAFQAQQByAHIAYQB5ACwAbQBhAHgAUABFAFQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAD4APQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApADwAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAD4APQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApADwAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQA+AD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQA8AD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAD4APQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAPAA9AG0AYQBwAF8AcABlAHQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABQAEUAVABBAHIAcgBhAHkAKQA+AD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAPAA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAD4APQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABJAHQAZQBtAEEAcgByAGEAeQAsACAAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAQwByAGkAdABlAHIAaQBhADEALAAgAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5ACwAIABRAHUAYQBuAHQAaQB0AHkALAAgAFsATQB1AGwAdABpAHAAbABpAGUAcgBdACwAIABbAEMAcgBpAHQAZQByAGkAYQAyAF0ALABbAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQBdACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgATQB1AGwAdABpAHAAbABpAGUAcgApACwAMQAsAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsAFwAbgAgACAAIAAgAHEAdQBhAG4AdABpAHQAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACoATQB1AGwAdABpAHAAbABpAGUAcgAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMQApACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADIALABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAcgBpAHQAZQByAGkAYQAyACkALAAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADIAKQApACwAXABuACAAIAAgACAAUwBVAE0AUABSAE8ARABVAEMAVAAoAGMAcgBpAHQAZQByAGkAYQAxACoAYwByAGkAdABlAHIAaQBhADIAKgBxAHUAYQBuAHQAaQB0AHkAKQBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApADwAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AJwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAG4AZQB4AHQAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPABTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAD4ARQApACwAXABuACAAIAAgACAAIAAgACAAIABuACwATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAcgBzACwAUwBFAFEAVQBFAE4AQwBFACgAbgAsADEALABmAGkAcgBzAHQAWQBlAGEAcgAsADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMALABEAEEAVABFACgAeQByAHMALABtACwAZAApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzACwATQBBAFAAKABzAHQAYQByAHQAcwAsAFAAZQByAGkAbwBkAEUAbgBkACkALABcAG4AIAAgACAAIAAgACAAIAAgAHQAYQBnACwASQBGACgAcwB0AGEAcgB0AHMAPQBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXAAiACAAKABUAGgAaQBzACAAcgBlAHAAbwByAHQAaQBuAGcAIABjAHkAYwBsAGUAKQBcACIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzAFQAZQB4AHQALABUAEUAWABUACgAcwB0AGEAcgB0AHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzAFQAZQB4AHQALABUAEUAWABUACgAZQBuAGQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgACYAIABcACIAIAB0AG8AIABcACIAIAAmACAAZQBuAGQAcwBUAGUAeAB0ACAAJgAgAHQAYQBnACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQBcAG4APQBMAEEATQBCAEQAQQAoAEYAdQBuAGMAdABpAG8AbgAsACAAVABFAFgAVABCAEUARgBPAFIARQAoAEYATwBSAE0AVQBMAEEAVABFAFgAVAAoAEYAdQBuAGMAdABpAG8AbgApACwAIABcACIAKABcACIAKQApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5ACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkALABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAA9AFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACAAPQAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5AD0AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkAPQBJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkAPQBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAD4AMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAJwBcACIAIAAmACAAcwBoACAAJgAgAFwAIgAnACEAXAAiACAAJgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEkATgAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBYACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAE0ATQBTACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -7227,22 +7227,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAG4AZAAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIAByAGUAdAB1AHIAbgBlAGQAIAB0AG8AIAB0AGgAZQAgAHMAbwBpAGwAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUARgBOAGkAIAAmACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAJgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAPAB0AD4APABzAD4AXAAiACAAJgBcAG4AIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFMAVQBCAFMAVABJAFQAVQBUAEUAKABDAGUAbABsACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEALABcACIAXAAiACkALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABEAGUAbABpAG0AaQB0AGUAcgAsAFwAIgA8AC8AcwA+ADwAcwA+AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAXAAiADwALwBzAD4APAAvAHQAPgBcACIALABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAvAC8AcwBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAGEAdgBnAFQAZQBtAHAALABhAHYAZwBSAGEAaQBuACwAZgByAG8AcwB0AEQAYQB5AHMALABlAGwAZQB2ACwAbQBhAHAAXwBwAGUAdAAsAFwAbgAgACAAIAAgAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACwAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkALABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUABFAFQAQQByAHIAYQB5ACwAbQBhAHgAUABFAFQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAD4APQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApADwAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAD4APQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApADwAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQA+AD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQA8AD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAD4APQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAPAA9AG0AYQBwAF8AcABlAHQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABQAEUAVABBAHIAcgBhAHkAKQA+AD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAPAA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAD4APQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABJAHQAZQBtAEEAcgByAGEAeQAsACAAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAQwByAGkAdABlAHIAaQBhADEALAAgAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5ACwAIABRAHUAYQBuAHQAaQB0AHkALAAgAFsATQB1AGwAdABpAHAAbABpAGUAcgBdACwAIABbAEMAcgBpAHQAZQByAGkAYQAyAF0ALABbAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQBdACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgATQB1AGwAdABpAHAAbABpAGUAcgApACwAMQAsAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsAFwAbgAgACAAIAAgAHEAdQBhAG4AdABpAHQAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACoATQB1AGwAdABpAHAAbABpAGUAcgAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMQApACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADIALABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAcgBpAHQAZQByAGkAYQAyACkALAAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADIAKQApACwAXABuACAAIAAgACAAUwBVAE0AUABSAE8ARABVAEMAVAAoAGMAcgBpAHQAZQByAGkAYQAxACoAYwByAGkAdABlAHIAaQBhADIAKgBxAHUAYQBuAHQAaQB0AHkAKQBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApADwAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AJwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAG4AZQB4AHQAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPABTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAD4ARQApACwAXABuACAAIAAgACAAIAAgACAAIABuACwATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAcgBzACwAUwBFAFEAVQBFAE4AQwBFACgAbgAsADEALABmAGkAcgBzAHQAWQBlAGEAcgAsADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMALABEAEEAVABFACgAeQByAHMALABtACwAZAApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzACwATQBBAFAAKABzAHQAYQByAHQAcwAsAFAAZQByAGkAbwBkAEUAbgBkACkALABcAG4AIAAgACAAIAAgACAAIAAgAHQAYQBnACwASQBGACgAcwB0AGEAcgB0AHMAPQBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXAAiACAAKABUAGgAaQBzACAAcgBlAHAAbwByAHQAaQBuAGcAIABjAHkAYwBsAGUAKQBcACIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzAFQAZQB4AHQALABUAEUAWABUACgAcwB0AGEAcgB0AHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzAFQAZQB4AHQALABUAEUAWABUACgAZQBuAGQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgACYAIABcACIAIAB0AG8AIABcACIAIAAmACAAZQBuAGQAcwBUAGUAeAB0ACAAJgAgAHQAYQBnACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQBcAG4APQBMAEEATQBCAEQAQQAoAEYAdQBuAGMAdABpAG8AbgAsACAAVABFAFgAVABCAEUARgBPAFIARQAoAEYATwBSAE0AVQBMAEEAVABFAFgAVAAoAEYAdQBuAGMAdABpAG8AbgApACwAIABcACIAKABcACIAKQApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5ACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkALABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAA9AFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACAAPQAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5AD0AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkAPQBJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkAPQBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAD4AMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAJwBcACIAIAAmACAAcwBoACAAJgAgAFwAIgAnACEAXAAiACAAJgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEkATgAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBYACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAE0ATQBTACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7261,18 +7246,29 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
finish scope 3 build, auto build left hand menu
</commit_message>
<xml_diff>
--- a/Excel/Common_v02.xlsx
+++ b/Excel/Common_v02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{077AD750-F2B3-4287-B715-9DC71F37E809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3430512-7572-48CA-91FD-562D441C3187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1350" yWindow="360" windowWidth="36255" windowHeight="19140" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="4680" yWindow="4680" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="3" r:id="rId1"/>
@@ -300,7 +300,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="69">
   <si>
     <t>Climate zone</t>
   </si>
@@ -505,6 +505,9 @@
   <si>
     <t>EFNi &amp; EFN2Oi</t>
   </si>
+  <si>
+    <t>APPENDICES</t>
+  </si>
 </sst>
 </file>
 
@@ -517,7 +520,7 @@
     <numFmt numFmtId="167" formatCode="[$-C09]dd\-mmmm\-yyyy;@"/>
     <numFmt numFmtId="168" formatCode="#,##0.000000"/>
   </numFmts>
-  <fonts count="32" x14ac:knownFonts="1">
+  <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -727,6 +730,20 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF404040"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -863,7 +880,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="59">
+  <cellStyleXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1029,8 +1046,9 @@
     <xf numFmtId="0" fontId="31" fillId="4" borderId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="26" fillId="4" borderId="0" xfId="8">
       <alignment horizontal="left" vertical="center"/>
@@ -1070,8 +1088,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="59"/>
+    <xf numFmtId="0" fontId="33" fillId="9" borderId="3" xfId="34" applyFont="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="33">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" xfId="35">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="59">
+  <cellStyles count="60">
     <cellStyle name="Block heading" xfId="5" xr:uid="{74527274-3B4A-494A-B37C-EA50686E114C}"/>
     <cellStyle name="Block subheading" xfId="47" xr:uid="{34E62905-A3E0-4883-B81A-BDB58FC88DA7}"/>
     <cellStyle name="Code" xfId="24" xr:uid="{99B3520F-01DD-4F8E-A8D0-24EAA04E90EB}"/>
@@ -1083,6 +1111,7 @@
     <cellStyle name="Equation source" xfId="6" xr:uid="{348FC12D-3392-478F-B0B3-D4FA4BBA59E4}"/>
     <cellStyle name="Equation table header" xfId="1" xr:uid="{11780056-D3CA-48D4-90AF-8DF1A50E1B13}"/>
     <cellStyle name="Euqation table row 2" xfId="13" xr:uid="{2CAEAB93-BC87-4606-B5A1-3C2F7B5C52A1}"/>
+    <cellStyle name="Hyperlink" xfId="59" builtinId="8"/>
     <cellStyle name="Information tip" xfId="39" xr:uid="{7D200D09-32E3-4546-9822-1B93AD118A74}"/>
     <cellStyle name="Information variation" xfId="54" xr:uid="{205494A3-14DD-4E6A-BDD3-5C5A864D6FA7}"/>
     <cellStyle name="Input block subheading" xfId="30" xr:uid="{A9FEBDB0-0992-4E30-96E5-9F9CAE92E3FB}"/>
@@ -3018,12 +3047,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76A159CA-1C38-4131-B0D4-3DBCDED3299D}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="str">
+        <f>HYPERLINK("#'Home'!A1", "Home")</f>
+        <v>Home</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="str">
+        <f>HYPERLINK("#'Constants - Common'!A1", "Constants - Common")</f>
+        <v>Constants - Common</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="str">
+        <f>HYPERLINK("#'Acknowledgements'!A1", "Acknowledgements")</f>
+        <v>Acknowledgements</v>
       </c>
     </row>
   </sheetData>
@@ -3067,9 +3119,14 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:65" s="8" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:65" s="8" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2"/>
+    </row>
     <row r="3" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3"/>
+      <c r="A3" s="17" t="str">
+        <f>HYPERLINK("#'Home'!A1", "Home")</f>
+        <v>Home</v>
+      </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -3105,7 +3162,9 @@
       <c r="BM5" s="2"/>
     </row>
     <row r="6" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6"/>
+      <c r="A6" s="16" t="s">
+        <v>68</v>
+      </c>
       <c r="D6" s="11" t="s">
         <v>1</v>
       </c>
@@ -3117,7 +3176,10 @@
       </c>
     </row>
     <row r="7" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7"/>
+      <c r="A7" s="18" t="str">
+        <f>HYPERLINK("#'Constants - Common'!A1", "Constants - Common")</f>
+        <v>Constants - Common</v>
+      </c>
       <c r="D7" s="11" t="str" cm="1">
         <f t="array" ref="D7">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</f>
         <v>New South Wales</v>
@@ -3132,7 +3194,10 @@
       </c>
     </row>
     <row r="8" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8"/>
+      <c r="A8" s="17" t="str">
+        <f>HYPERLINK("#'Acknowledgements'!A1", "Acknowledgements")</f>
+        <v>Acknowledgements</v>
+      </c>
       <c r="D8" s="11" t="str" cm="1">
         <f t="array" ref="D8">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</f>
         <v>Australian Capital Territory</v>
@@ -3425,6 +3490,7 @@
       </c>
     </row>
     <row r="42" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42"/>
       <c r="D42" s="11" t="str" cm="1">
         <f t="array" ref="D42">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</f>
         <v>SF6</v>
@@ -3435,6 +3501,7 @@
       </c>
     </row>
     <row r="43" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43"/>
       <c r="D43" s="11" t="str" cm="1">
         <f t="array" ref="D43">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</f>
         <v>NF3</v>
@@ -3444,20 +3511,25 @@
         <v>17200</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44"/>
+    </row>
     <row r="45" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45"/>
       <c r="D45" s="5" t="str" cm="1">
         <f t="array" ref="D45">Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Title()</f>
         <v>Factor to convert elemental mass of gas to molecular mass</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46"/>
       <c r="D46" s="4" t="str" cm="1">
         <f t="array" ref="D46">Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Source()</f>
         <v>XXXXXXX</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47"/>
       <c r="D47" s="11" t="s">
         <v>5</v>
       </c>
@@ -3475,6 +3547,7 @@
       </c>
     </row>
     <row r="48" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48"/>
       <c r="D48" s="11" t="str" cm="1">
         <f t="array" ref="D48">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
         <v>CO2</v>
@@ -3496,7 +3569,8 @@
         <v>3.6666666666666665</v>
       </c>
     </row>
-    <row r="49" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49"/>
       <c r="D49" s="11" t="str" cm="1">
         <f t="array" ref="D49">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
         <v>CH4</v>
@@ -3518,7 +3592,8 @@
         <v>1.3333333333333333</v>
       </c>
     </row>
-    <row r="50" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50"/>
       <c r="D50" s="11" t="str" cm="1">
         <f t="array" ref="D50">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
         <v>N2O</v>
@@ -3540,7 +3615,8 @@
         <v>1.5714285714285714</v>
       </c>
     </row>
-    <row r="51" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51"/>
       <c r="D51" s="11" t="str" cm="1">
         <f t="array" ref="D51">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
         <v>Nox</v>
@@ -3562,7 +3638,8 @@
         <v>3.2857142857142856</v>
       </c>
     </row>
-    <row r="52" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52"/>
       <c r="D52" s="11" t="str" cm="1">
         <f t="array" ref="D52">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
         <v>CO</v>
@@ -3584,7 +3661,8 @@
         <v>2.3333333333333335</v>
       </c>
     </row>
-    <row r="53" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53"/>
       <c r="D53" s="11" t="str" cm="1">
         <f t="array" ref="D53">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
         <v>CO2 Lime</v>
@@ -3606,7 +3684,8 @@
         <v>3.6666666666666665</v>
       </c>
     </row>
-    <row r="54" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54"/>
       <c r="D54" s="11" t="str" cm="1">
         <f t="array" ref="D54">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
         <v>NMVOC</v>
@@ -3628,38 +3707,50 @@
         <v>1.1666666666666667</v>
       </c>
     </row>
-    <row r="55" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55"/>
+    </row>
+    <row r="56" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56"/>
+    </row>
+    <row r="57" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57"/>
       <c r="D57" s="5" t="str" cm="1">
         <f t="array" ref="D57">Common_SourceData.Common_SourceData_WetAndDryZones_Title()</f>
         <v>VEERG Australian wet and dry zones</v>
       </c>
     </row>
-    <row r="58" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58"/>
       <c r="D58" s="4" t="str" cm="1">
         <f t="array" ref="D58">Common_SourceData.Common_SourceData_WetAndDryZones_Source()</f>
         <v>VEERG 2026: Table 1.2: Translating climate zones to wet and dry zones</v>
       </c>
     </row>
-    <row r="59" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59"/>
       <c r="D59" s="13" t="str" cm="1">
         <f t="array" ref="D59:D61">"⚠️" &amp; Common_SourceData.Common_SourceData_WetAndDryZones_Variation()</f>
         <v>⚠️VARIATION OF SOURCE DATA:</v>
       </c>
     </row>
-    <row r="60" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60"/>
       <c r="D60" s="13" t="str">
         <v>⚠️Added warm / cool temperate moist / dry - low frost and high temp classes to accommodate climate scenarios excluded by VEERG criteria.</v>
       </c>
     </row>
-    <row r="61" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61"/>
       <c r="D61" s="13" t="str">
         <v>⚠️Fixed typo - Changed 'Fry' to 'Dry'.</v>
       </c>
     </row>
-    <row r="62" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62"/>
+    </row>
+    <row r="63" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63"/>
       <c r="D63" s="11" t="s">
         <v>0</v>
       </c>
@@ -3667,7 +3758,8 @@
         <v>23</v>
       </c>
     </row>
-    <row r="64" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64"/>
       <c r="D64" s="11" t="str" cm="1">
         <f t="array" ref="D64">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Tropical montane</v>
@@ -3677,7 +3769,8 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="65" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65"/>
       <c r="D65" s="11" t="str" cm="1">
         <f t="array" ref="D65">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Tropical wet</v>
@@ -3687,7 +3780,8 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="66" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66"/>
       <c r="D66" s="11" t="str" cm="1">
         <f t="array" ref="D66">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Tropical moist</v>
@@ -3697,7 +3791,8 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="67" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67"/>
       <c r="D67" s="11" t="str" cm="1">
         <f t="array" ref="D67">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Tropical dry</v>
@@ -3707,7 +3802,8 @@
         <v>Dry climate zone</v>
       </c>
     </row>
-    <row r="68" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68"/>
       <c r="D68" s="11" t="str" cm="1">
         <f t="array" ref="D68">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Warm temperate moist</v>
@@ -3717,7 +3813,8 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="69" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69"/>
       <c r="D69" s="11" t="str" cm="1">
         <f t="array" ref="D69">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Warm temperate dry</v>
@@ -3727,7 +3824,8 @@
         <v>Dry climate zone</v>
       </c>
     </row>
-    <row r="70" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70"/>
       <c r="D70" s="11" t="str" cm="1">
         <f t="array" ref="D70">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Cool temperate moist</v>
@@ -3737,7 +3835,8 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="71" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71"/>
       <c r="D71" s="11" t="str" cm="1">
         <f t="array" ref="D71">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Cool temperate dry</v>
@@ -3747,7 +3846,8 @@
         <v>Dry climate zone</v>
       </c>
     </row>
-    <row r="72" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A72"/>
       <c r="D72" s="11" t="str" cm="1">
         <f t="array" ref="D72">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Warm temperate moist - low frost</v>
@@ -3757,7 +3857,8 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="73" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A73"/>
       <c r="D73" s="11" t="str" cm="1">
         <f t="array" ref="D73">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Warm temperate dry - low frost</v>
@@ -3767,7 +3868,8 @@
         <v>Dry climate zone</v>
       </c>
     </row>
-    <row r="74" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74"/>
       <c r="D74" s="11" t="str" cm="1">
         <f t="array" ref="D74">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Warm temperate moist - high temp</v>
@@ -3777,7 +3879,8 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="75" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75"/>
       <c r="D75" s="11" t="str" cm="1">
         <f t="array" ref="D75">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Warm temperate dry - high temp</v>
@@ -3787,7 +3890,8 @@
         <v>Dry climate zone</v>
       </c>
     </row>
-    <row r="76" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76"/>
       <c r="D76" s="11" t="str" cm="1">
         <f t="array" ref="D76">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Cool temperate moist - low frost</v>
@@ -3797,7 +3901,8 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="77" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77"/>
       <c r="D77" s="11" t="str" cm="1">
         <f t="array" ref="D77">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
         <v>Cool temperate dry - low frost</v>
@@ -3807,49 +3912,65 @@
         <v>Dry climate zone</v>
       </c>
     </row>
-    <row r="78" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78"/>
+    </row>
+    <row r="79" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79"/>
+    </row>
+    <row r="80" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80"/>
+    </row>
+    <row r="81" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81"/>
       <c r="D81" s="5" t="str" cm="1">
         <f t="array" ref="D81">Common_SourceData.Common_SourceData_ClimateZones_Title()</f>
         <v>VEERG Australian climate zones</v>
       </c>
     </row>
-    <row r="82" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A82"/>
       <c r="D82" s="4" t="str" cm="1">
         <f t="array" ref="D82">Common_SourceData.Common_SourceData_ClimateZones_Source()</f>
         <v>VEERG 2026: Table 1.3: Climate and Rainfall zone classifications and definitions</v>
       </c>
     </row>
-    <row r="83" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A83"/>
       <c r="D83" s="13" t="str" cm="1">
         <f t="array" ref="D83:D87">"⚠️" &amp; Common_SourceData.Common_SourceData_ClimateZones_Variation()</f>
         <v>⚠️VARIATION OF SOURCE DATA:</v>
       </c>
     </row>
-    <row r="84" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A84"/>
       <c r="D84" s="13" t="str">
         <v>⚠️Added warm / cool temperate moist / dry - low frost and high temp classes to accommodate climate scenarios excluded by VEERG criteria.</v>
       </c>
     </row>
-    <row r="85" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A85"/>
       <c r="D85" s="13" t="str">
         <v>⚠️Fixed typo in MAT value for warm temperate dry - changed 10 to 11.</v>
       </c>
     </row>
-    <row r="86" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A86"/>
       <c r="D86" s="13" t="str">
         <v>⚠️Added min and max columns for MAT, MAP, frost days per year, elevation, MAP:PET to calculate zones from real climate data.</v>
       </c>
     </row>
-    <row r="87" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A87"/>
       <c r="D87" s="13" t="str">
         <v>⚠️GAF accepts rainfall as a proxy for precipitation.</v>
       </c>
     </row>
-    <row r="88" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A88"/>
+    </row>
+    <row r="89" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A89"/>
       <c r="D89" s="11" t="s">
         <v>0</v>
       </c>
@@ -3900,7 +4021,8 @@
       </c>
       <c r="T89" s="11"/>
     </row>
-    <row r="90" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90"/>
       <c r="D90" s="11" t="str" cm="1">
         <f t="array" ref="D90">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
         <v>Tropical montane</v>
@@ -3967,7 +4089,8 @@
       </c>
       <c r="T90" s="11"/>
     </row>
-    <row r="91" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A91"/>
       <c r="D91" s="11" t="str" cm="1">
         <f t="array" ref="D91">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
         <v>Tropical wet</v>
@@ -4034,7 +4157,8 @@
       </c>
       <c r="T91" s="11"/>
     </row>
-    <row r="92" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A92"/>
       <c r="D92" s="11" t="str" cm="1">
         <f t="array" ref="D92">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
         <v>Tropical moist</v>
@@ -4101,7 +4225,8 @@
       </c>
       <c r="T92" s="11"/>
     </row>
-    <row r="93" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A93"/>
       <c r="D93" s="11" t="str" cm="1">
         <f t="array" ref="D93">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
         <v>Tropical dry</v>
@@ -4168,7 +4293,8 @@
       </c>
       <c r="T93" s="11"/>
     </row>
-    <row r="94" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A94"/>
       <c r="D94" s="11" t="str" cm="1">
         <f t="array" ref="D94">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
         <v>Warm temperate moist</v>
@@ -4235,7 +4361,8 @@
       </c>
       <c r="T94" s="11"/>
     </row>
-    <row r="95" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A95"/>
       <c r="D95" s="11" t="str" cm="1">
         <f t="array" ref="D95">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
         <v>Warm temperate dry</v>
@@ -4302,7 +4429,8 @@
       </c>
       <c r="T95" s="11"/>
     </row>
-    <row r="96" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A96"/>
       <c r="D96" s="11" t="str" cm="1">
         <f t="array" ref="D96">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
         <v>Cool temperate moist</v>
@@ -4369,7 +4497,8 @@
       </c>
       <c r="T96" s="11"/>
     </row>
-    <row r="97" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97"/>
       <c r="D97" s="11" t="str" cm="1">
         <f t="array" ref="D97">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
         <v>Cool temperate dry</v>
@@ -4436,52 +4565,67 @@
       </c>
       <c r="T97" s="11"/>
     </row>
-    <row r="98" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A98"/>
+    </row>
+    <row r="99" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A99"/>
       <c r="D99" s="12" t="str" cm="1">
         <f t="array" ref="D99:D102">Common_SourceData.Common_SourceData_ClimateZones_Appendices()</f>
         <v>Note:</v>
       </c>
     </row>
-    <row r="100" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A100"/>
       <c r="D100" s="12" t="str">
         <v>MAT = mean annual temperature</v>
       </c>
     </row>
-    <row r="101" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A101"/>
       <c r="D101" s="12" t="str">
         <v>MAP = mean annual precipitation</v>
       </c>
     </row>
-    <row r="102" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A102"/>
       <c r="D102" s="12" t="str">
         <v>PET = potential evapotranspiration</v>
       </c>
     </row>
-    <row r="103" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A103"/>
       <c r="D103" s="12"/>
     </row>
-    <row r="104" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A104"/>
+    </row>
+    <row r="105" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A105"/>
       <c r="D105" s="5" t="str" cm="1">
         <f t="array" ref="D105">Common_SourceData.Common_SourceData_TemperatureZones_Title()</f>
         <v>VEERG Australian temperature zones</v>
       </c>
     </row>
-    <row r="106" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A106"/>
       <c r="D106" s="4" t="str" cm="1">
         <f t="array" ref="D106">Common_SourceData.Common_SourceData_TemperatureZones_Source()</f>
         <v>VEERG 2026: Table 1.3: Climate and Rainfall zone classifications and definitions</v>
       </c>
     </row>
-    <row r="107" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A107"/>
       <c r="D107" s="13" t="str" cm="1">
         <f t="array" ref="D107">"⚠️" &amp; Common_SourceData.Common_SourceData_TemperatureZones_Variation()</f>
         <v>⚠️VARIATION OF SOURCE DATA: Added extra MAT min and MAT max columns to calculate zone from real temperature data.</v>
       </c>
     </row>
-    <row r="108" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A108"/>
+    </row>
+    <row r="109" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A109"/>
       <c r="D109" s="11" t="s">
         <v>27</v>
       </c>
@@ -4495,7 +4639,8 @@
         <v>29</v>
       </c>
     </row>
-    <row r="110" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A110"/>
       <c r="D110" s="11" t="str" cm="1">
         <f t="array" ref="D110">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</f>
         <v>Warm</v>
@@ -4513,7 +4658,8 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="111" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A111"/>
       <c r="D111" s="11" t="str" cm="1">
         <f t="array" ref="D111">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</f>
         <v>Temperate</v>
@@ -4531,7 +4677,8 @@
         <v>25.998999999999999</v>
       </c>
     </row>
-    <row r="112" spans="4:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A112"/>
       <c r="D112" s="11" t="str" cm="1">
         <f t="array" ref="D112">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</f>
         <v>Cool</v>
@@ -4549,33 +4696,42 @@
         <v>14.999000000000001</v>
       </c>
     </row>
-    <row r="113" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A113"/>
+    </row>
+    <row r="114" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A114"/>
+    </row>
+    <row r="115" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A115"/>
       <c r="D115" s="5" t="str" cm="1">
         <f t="array" ref="D115">Common_SourceData.Common_SourceData_RainfallZones_Title()</f>
         <v>VEERG Australian rainfall zones</v>
       </c>
       <c r="BN115" s="6"/>
     </row>
-    <row r="116" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A116"/>
       <c r="D116" s="4" t="str" cm="1">
         <f t="array" ref="D116">Common_SourceData.Common_SourceData_RainfallZones_Source()</f>
         <v>VEERG 2026: Table 1.3: Climate and Rainfall zone classifications and definitions</v>
       </c>
       <c r="BN116" s="6"/>
     </row>
-    <row r="117" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A117"/>
       <c r="D117" s="13" t="str" cm="1">
         <f t="array" ref="D117">"⚠️" &amp; Common_SourceData.Common_SourceData_RainfallZones_Variation()</f>
         <v>⚠️VARIATION OF SOURCE DATA: Added extra Rainfall min and Rainfall max columns to calculate zone from real rainfall data.</v>
       </c>
       <c r="BN117" s="6"/>
     </row>
-    <row r="118" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A118"/>
       <c r="BN118" s="6"/>
     </row>
-    <row r="119" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A119"/>
       <c r="D119" s="11" t="s">
         <v>30</v>
       </c>
@@ -4590,7 +4746,8 @@
       </c>
       <c r="BN119" s="6"/>
     </row>
-    <row r="120" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A120"/>
       <c r="D120" s="11" t="str" cm="1">
         <f t="array" ref="D120">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</f>
         <v>High rainfall</v>
@@ -4609,7 +4766,8 @@
       </c>
       <c r="BN120" s="6"/>
     </row>
-    <row r="121" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A121"/>
       <c r="D121" s="11" t="str" cm="1">
         <f t="array" ref="D121">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</f>
         <v>Low rainfall</v>
@@ -4628,24 +4786,32 @@
       </c>
       <c r="BN121" s="6"/>
     </row>
-    <row r="122" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A122"/>
       <c r="BN122" s="6"/>
     </row>
-    <row r="123" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A123"/>
+    </row>
+    <row r="124" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A124"/>
       <c r="D124" s="5" t="str" cm="1">
         <f t="array" ref="D124">Common_SourceData.Common_SourceData_LeachingZones_Title()</f>
         <v>VEERG Australian leaching zones</v>
       </c>
     </row>
-    <row r="125" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A125"/>
       <c r="D125" s="4" t="str" cm="1">
         <f t="array" ref="D125">Common_SourceData.Common_SourceData_LeachingZones_Source()</f>
         <v>VEERG 2026: Table 1.3: Climate and Rainfall zone classifications and definitions</v>
       </c>
     </row>
-    <row r="126" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A126"/>
+    </row>
+    <row r="127" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A127"/>
       <c r="D127" s="11" t="s">
         <v>32</v>
       </c>
@@ -4653,7 +4819,8 @@
         <v>33</v>
       </c>
     </row>
-    <row r="128" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A128"/>
       <c r="D128" s="11" t="str" cm="1">
         <f t="array" ref="D128">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</f>
         <v>Leaching occurs</v>
@@ -4663,7 +4830,8 @@
         <v>Σ(𝑟𝑎𝑖𝑛)&gt;Σ(𝐸𝑇0)+𝑠𝑜𝑖𝑙 𝑤𝑎𝑡𝑒𝑟 ℎ𝑜𝑙𝑑𝑖𝑛𝑔 𝑐𝑎𝑝𝑎𝑐𝑖𝑡𝑦</v>
       </c>
     </row>
-    <row r="129" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A129"/>
       <c r="D129" s="11" t="str" cm="1">
         <f t="array" ref="D129">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</f>
         <v>Leaching does not occur</v>
@@ -4673,23 +4841,30 @@
         <v>Σ(𝑟𝑎𝑖𝑛)≤Σ(𝐸𝑇0)+𝑠𝑜𝑖𝑙 𝑤𝑎𝑡𝑒𝑟 ℎ𝑜𝑙𝑑𝑖𝑛𝑔 𝑐𝑎𝑝𝑎𝑐𝑖𝑡𝑦</v>
       </c>
     </row>
-    <row r="130" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A130"/>
+    </row>
+    <row r="131" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A131"/>
+    </row>
+    <row r="132" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A132"/>
       <c r="D132" s="5" t="str" cm="1">
         <f t="array" ref="D132">Common_SourceData.Common_SourceData_FracWET_Title()</f>
         <v>Fraction of N that is available for leaching and runoff</v>
       </c>
       <c r="E132" s="10"/>
     </row>
-    <row r="133" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A133"/>
       <c r="D133" s="4" t="str" cm="1">
         <f t="array" ref="D133">Common_SourceData.Common_SourceData_FracWET_Source()</f>
         <v>VEERG 2026:5.5.2.3 Constant Parameters</v>
       </c>
       <c r="E133" s="10"/>
     </row>
-    <row r="134" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A134"/>
       <c r="D134" t="s">
         <v>37</v>
       </c>
@@ -4697,7 +4872,8 @@
         <v>38</v>
       </c>
     </row>
-    <row r="135" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A135"/>
       <c r="D135" t="str" cm="1">
         <f t="array" ref="D135">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</f>
         <v>Yes - in leaching zone</v>
@@ -4707,7 +4883,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A136"/>
       <c r="D136" s="1" t="str" cm="1">
         <f t="array" ref="D136">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</f>
         <v>No - not in leaching zone</v>
@@ -4717,8 +4894,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A137"/>
+    </row>
+    <row r="138" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A138"/>
       <c r="BN138" s="6"/>
       <c r="BO138" s="6"/>
       <c r="BP138" s="6"/>
@@ -4732,7 +4912,8 @@
       <c r="BX138" s="6"/>
       <c r="BY138" s="6"/>
     </row>
-    <row r="139" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A139"/>
       <c r="D139" s="5" t="str" cm="1">
         <f t="array" ref="D139">Common_SourceData.Common_SourceData_FracWETIrrigation_Title()</f>
         <v>FracWET for irrigation types</v>
@@ -4750,7 +4931,8 @@
       <c r="BX139" s="6"/>
       <c r="BY139" s="6"/>
     </row>
-    <row r="140" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A140"/>
       <c r="D140" s="4" t="str" cm="1">
         <f t="array" ref="D140">Common_SourceData.Common_SourceData_FracWETIrrigation_Source()</f>
         <v>VEERG 2026: Chapter 1, section 1.8.2 Leaching, climate and rainfall zones</v>
@@ -4768,14 +4950,16 @@
       <c r="BX140" s="6"/>
       <c r="BY140" s="6"/>
     </row>
-    <row r="141" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A141"/>
       <c r="D141" s="13" t="str" cm="1">
         <f t="array" ref="D141">Common_SourceData.Common_SourceData_FracWETIrrigation_Variation()</f>
         <v>VARIATION FROM SOURCE DATA: Table created based on VEERG text 'Areas are subject to leaching (i.e., in the leaching zone) when... the land is irrigated (except drip irrigation).'</v>
       </c>
       <c r="BN141" s="6"/>
     </row>
-    <row r="142" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A142"/>
       <c r="D142" s="11" t="s">
         <v>46</v>
       </c>
@@ -4784,7 +4968,8 @@
       </c>
       <c r="BN142" s="6"/>
     </row>
-    <row r="143" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A143"/>
       <c r="D143" s="11" t="str" cm="1">
         <f t="array" ref="D143">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</f>
         <v>Not irrigated</v>
@@ -4795,7 +4980,8 @@
       </c>
       <c r="BN143" s="6"/>
     </row>
-    <row r="144" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A144"/>
       <c r="D144" s="1" t="str" cm="1">
         <f t="array" ref="D144">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</f>
         <v>Drip irrigation</v>
@@ -4806,7 +4992,8 @@
       </c>
       <c r="BN144" s="6"/>
     </row>
-    <row r="145" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A145"/>
       <c r="D145" s="1" t="str" cm="1">
         <f t="array" ref="D145">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</f>
         <v>Sprinkler irrigation</v>
@@ -4817,7 +5004,8 @@
       </c>
       <c r="BN145" s="6"/>
     </row>
-    <row r="146" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A146"/>
       <c r="D146" s="1" t="str" cm="1">
         <f t="array" ref="D146">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</f>
         <v>Surface irrigation</v>
@@ -4828,7 +5016,8 @@
       </c>
       <c r="BN146" s="6"/>
     </row>
-    <row r="147" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A147"/>
       <c r="D147" s="1" t="str" cm="1">
         <f t="array" ref="D147">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</f>
         <v>Other irrigation</v>
@@ -4839,30 +5028,36 @@
       </c>
       <c r="BN147" s="6"/>
     </row>
-    <row r="148" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A148"/>
       <c r="BN148" s="6"/>
     </row>
-    <row r="149" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A149"/>
       <c r="BN149" s="6"/>
     </row>
-    <row r="150" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A150"/>
       <c r="D150" s="5" t="str" cm="1">
         <f t="array" ref="D150">Common_SourceData.Common_SourceData_DataScores_Scope3_Title()</f>
         <v>Australian data scores for scope 3</v>
       </c>
       <c r="BN150" s="6"/>
     </row>
-    <row r="151" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A151"/>
       <c r="D151" s="4" t="str" cm="1">
         <f t="array" ref="D151">Common_SourceData.Common_SourceData_DataScores_Scope3_Source()</f>
         <v>VEERG 2026: XXXXXXXX</v>
       </c>
       <c r="BN151" s="6"/>
     </row>
-    <row r="152" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A152"/>
       <c r="BN152" s="6"/>
     </row>
-    <row r="153" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A153"/>
       <c r="D153" s="11" t="s">
         <v>34</v>
       </c>
@@ -4881,7 +5076,8 @@
       <c r="BL153" s="2"/>
       <c r="BM153" s="2"/>
     </row>
-    <row r="154" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A154"/>
       <c r="D154" s="11" t="str" cm="1">
         <f t="array" ref="D154">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
         <v>International scope 3 database</v>
@@ -4902,7 +5098,8 @@
       <c r="BL154" s="2"/>
       <c r="BM154" s="2"/>
     </row>
-    <row r="155" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A155"/>
       <c r="D155" s="11" t="str" cm="1">
         <f t="array" ref="D155">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
         <v>Australian scope 3 database</v>
@@ -4923,7 +5120,8 @@
       <c r="BL155" s="2"/>
       <c r="BM155" s="2"/>
     </row>
-    <row r="156" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A156"/>
       <c r="D156" s="11" t="str" cm="1">
         <f t="array" ref="D156">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
         <v>State or regional scope 3 database</v>
@@ -4933,7 +5131,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="157" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A157"/>
       <c r="D157" s="11" t="str" cm="1">
         <f t="array" ref="D157">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
         <v>Emissions intensity calculated from approved method</v>
@@ -4943,7 +5142,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="158" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A158"/>
       <c r="D158" s="11" t="str" cm="1">
         <f t="array" ref="D158">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
         <v>Verified credential matching ISO14067</v>
@@ -4953,8 +5153,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="159" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="4:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A159"/>
+    </row>
+    <row r="160" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A160"/>
+    </row>
     <row r="161" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D161" s="5" t="str" cm="1">
         <f t="array" ref="D161">Common_SourceData.Common_SourceData_FracLEACH_Title()</f>
@@ -7025,12 +7229,35 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F00F8506-5EB7-47C9-955C-A68351EE5687}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="17" t="str">
+        <f>HYPERLINK("#'Home'!A1", "Home")</f>
+        <v>Home</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="str">
+        <f>HYPERLINK("#'Constants - Common'!A1", "Constants - Common")</f>
+        <v>Constants - Common</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="18" t="str">
+        <f>HYPERLINK("#'Acknowledgements'!A1", "Acknowledgements")</f>
+        <v>Acknowledgements</v>
       </c>
     </row>
   </sheetData>
@@ -7039,19 +7266,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -7246,6 +7460,19 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -7258,22 +7485,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7292,6 +7503,22 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>

</xml_diff>